<commit_message>
Changes made to incorporate shell-less data into optimization
</commit_message>
<xml_diff>
--- a/src/data/data_stat_new.xlsx
+++ b/src/data/data_stat_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/eric_cytrynbaum_ubc_ca/Documents/Documents/Research/GitHub/Cell-Chirality-Model/src/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chakradhar/Desktop/Cellular Chirality model/chirality_C_elegans_In_Vivo/src/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BC855E5-60A0-D241-BF2B-A84BEA386D82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA9E783-5F1A-424F-B78A-0DE54C579F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -49,29 +49,29 @@
     <t>ABp_ant_avg</t>
   </si>
   <si>
-    <t>ABa_dorsal_stdeofmean</t>
-  </si>
-  <si>
-    <t>ABp_dorsal_stdeofmean</t>
-  </si>
-  <si>
-    <t>ABa_ant_stdeofmean</t>
-  </si>
-  <si>
-    <t>ABp_ant_stdeofmean</t>
-  </si>
-  <si>
     <t>dorsal_t_test</t>
   </si>
   <si>
     <t>ant_t_test</t>
+  </si>
+  <si>
+    <t>ABa_dorsal_CIhalfwidth</t>
+  </si>
+  <si>
+    <t>ABp_dorsal_CIhalfwidth</t>
+  </si>
+  <si>
+    <t>ABa_ant_CIhalfwidth</t>
+  </si>
+  <si>
+    <t>ABp_ant_CIhalfwidth</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,6 +83,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -120,9 +126,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -446,23 +455,23 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>